<commit_message>
fixed cf4 generate errors. added optional time in the templates for cf2
</commit_message>
<xml_diff>
--- a/templates/CF2_Template.xlsx
+++ b/templates/CF2_Template.xlsx
@@ -1,152 +1,64 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Romel\Desktop\Projects\BeaconAutomation2\templates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85D9BEEE-EDCE-4390-9175-E0409997E908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="NyzUZmyJcBlqrKMF9zVLu3ig5pbohhQRBcZTlnP4vkHSElVb6X+OcEl3UPMU+fVPoLLDKXpg5VStCUPJn9w86Q==" workbookSaltValue="09mbXxWE4uMRCt1jx3au1w==" workbookSpinCount="100000" lockStructure="1"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection lockStructure="1" workbookAlgorithmName="SHA-512" workbookHashValue="NyzUZmyJcBlqrKMF9zVLu3ig5pbohhQRBcZTlnP4vkHSElVb6X+OcEl3UPMU+fVPoLLDKXpg5VStCUPJn9w86Q==" workbookSaltValue="09mbXxWE4uMRCt1jx3au1w==" workbookSpinCount="100000"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1942E4D1-440A-4CAB-9580-C5A30C9887D6}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$E$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>NAME OF PATIENT</t>
-  </si>
-  <si>
-    <t>ATTENDING/ NEPHROLOGIST</t>
-  </si>
-  <si>
-    <t>TREATMENT DATES</t>
-  </si>
-  <si>
-    <t>ACCREDITATION NO.</t>
-  </si>
-  <si>
-    <t>1202-0400315-0</t>
-  </si>
-  <si>
-    <t>JOSEPH FRANCIS B. ASTORGA</t>
-  </si>
-  <si>
-    <t>09352408339</t>
-  </si>
-  <si>
-    <t>A/R STAFF</t>
-  </si>
-  <si>
-    <t>LILIBETH B. IBARRIENTOS</t>
-  </si>
-  <si>
-    <t>JULY 1, 2, 3, 4</t>
-  </si>
-  <si>
-    <t>MEMBER PIN</t>
-  </si>
-  <si>
-    <t>MICAYAS, ROLEX S</t>
-  </si>
-  <si>
-    <t>10255010315/</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>NOTES:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> IF DEPENDENTS: ADD "/" AT THE END OF THE PIN EX: 10255010315/  USE ONLY THE MEMBER'S PIN NOT THE DEPENDENT'S PIN</t>
-    </r>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="5">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -165,64 +77,123 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="16">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -522,102 +493,140 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67DFE70F-ACDA-4E6F-BDC8-4401456305A7}">
-  <sheetPr codeName="Sheet1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr codeName="Sheet1">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultColWidth="21.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="21.28515625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="33.5703125" style="9" customWidth="1"/>
-    <col min="2" max="2" width="38" style="4" customWidth="1"/>
-    <col min="3" max="3" width="36.140625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="37" style="4" customWidth="1"/>
-    <col min="5" max="5" width="36.7109375" style="5" customWidth="1"/>
-    <col min="6" max="16384" width="21.28515625" style="4"/>
+    <col width="33.5703125" customWidth="1" style="9" min="1" max="1"/>
+    <col width="38" customWidth="1" style="12" min="2" max="2"/>
+    <col width="36.140625" customWidth="1" style="12" min="3" max="3"/>
+    <col width="37" customWidth="1" style="12" min="4" max="4"/>
+    <col width="36.7109375" customWidth="1" style="13" min="5" max="5"/>
+    <col width="24" customWidth="1" style="12" min="6" max="16384"/>
+    <col width="21.28515625" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="15" t="s">
-        <v>13</v>
+    <row r="1" ht="32.25" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>MEMBER PIN</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>NAME OF PATIENT</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>ATTENDING/ NEPHROLOGIST</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>ACCREDITATION NO.</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>TREATMENT DATES</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>TIME (OPTIONAL)</t>
+        </is>
+      </c>
+      <c r="G1" s="15" t="inlineStr">
+        <is>
+          <t>NOTES: IF DEPENDENTS: ADD "/" AT THE END OF THE PIN EX: 10255010315/  USE ONLY THE MEMBER'S PIN NOT THE DEPENDENT'S PIN</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" s="14"/>
+    <row r="2" customFormat="1" s="12">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>10255010315/</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>MICAYAS, ROLEX S</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>LILIBETH B. IBARRIENTOS</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>1202-0400315-0</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>JULY 1, 2, 3, 4</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr">
+        <is>
+          <t>05:25PM-09:25PM</t>
+        </is>
+      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G3" s="15"/>
+    <row r="3">
+      <c r="F3" s="15" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection formatCells="0" formatRows="0" insertRows="0" insertHyperlinks="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
-  <protectedRanges>
-    <protectedRange sqref="A1:E299" name="Range1" securityDescriptor="O:WDG:WDD:(A;;CC;;;WD)"/>
-  </protectedRanges>
-  <autoFilter ref="A1:E1" xr:uid="{67DFE70F-ACDA-4E6F-BDC8-4401456305A7}"/>
+  <autoFilter ref="A1:E1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94AC9A9A-891E-46BC-A907-4E54D6AAED6D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="31.28515625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" style="3" customWidth="1"/>
-    <col min="3" max="4" width="9.140625" style="3"/>
-    <col min="5" max="5" width="13" style="3" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="3"/>
+    <col width="31.28515625" customWidth="1" style="3" min="1" max="1"/>
+    <col width="11.5703125" customWidth="1" style="3" min="2" max="2"/>
+    <col width="9.140625" customWidth="1" style="3" min="3" max="4"/>
+    <col width="13" customWidth="1" style="3" min="5" max="5"/>
+    <col width="9.140625" customWidth="1" style="3" min="6" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>7</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>JOSEPH FRANCIS B. ASTORGA</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>A/R STAFF</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>6</v>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>09352408339</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
-  <protectedRanges>
-    <protectedRange sqref="A1:B2" name="Range1"/>
-  </protectedRanges>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>